<commit_message>
Close phase 3 portal test coverage
</commit_message>
<xml_diff>
--- a/docs_generali/Matrice_portali.xlsx
+++ b/docs_generali/Matrice_portali.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali esistenti" sheetId="1" r:id="R562d87e0396d4373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali candidati" sheetId="2" r:id="R595326112a0a4465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali esistenti" sheetId="1" r:id="R74293ec425ac473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali candidati" sheetId="2" r:id="R70264843059648eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -471,438 +471,507 @@
     </x:row>
     <x:row r="8" ht="132" hidden="0" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>bub_digitale</x:v>
+        <x:v>biblioteca_digitale_siena</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>BUB Digitale</x:v>
+        <x:v>Biblioteca Digitale Siena</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Italia / Emilia-Romagna</x:v>
+        <x:v>Italia / Toscana</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>IIIF diretto da parametro manifest= nelle pagine BUB</x:v>
+        <x:v>IIIF diretto da viewer item-level vieweriiif e manifest pubblico BDS</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
-        <x:v>Accesso libero per studio/ricerca; licenza e riuso da verificare per singolo oggetto</x:v>
+        <x:v>JPG web-resolution consentiti per uso personale, studio e ricerca; citazione BDS obbligatoria e uso commerciale escluso</x:v>
       </x:c>
       <x:c r="G8" s="10" t="str">
-        <x:v>Supportare solo manifest BUB pubblici, con range esplicito e avviso licenza item-level</x:v>
+        <x:v>Supportare solo manifest item-level pubblici BDS, con range esplicito, ritmo prudente e verifica delle condizioni del singolo oggetto</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="198" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>dl_ficlit</x:v>
+        <x:v>bub_digitale</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>FICLIT Digital Library</x:v>
+        <x:v>BUB Digitale</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>Italia / Emilia-Romagna</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>IIIF diretto da item Omeka S o manifest FICLIT; download da immagine diretta canvas</x:v>
+        <x:v>IIIF diretto da parametro manifest= nelle pagine BUB</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>Condizioni d'uso specifiche per item set/collezione; corretta citazione richiesta</x:v>
+        <x:v>Accesso libero per studio/ricerca; licenza e riuso da verificare per singolo oggetto</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
-        <x:v>Supportare solo item/manifest FICLIT pubblici, con range esplicito e verifica termini item-level; evitare tile service per HTTP 500 sui ritagli</x:v>
+        <x:v>Supportare solo manifest BUB pubblici, con range esplicito e avviso licenza item-level</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="198" hidden="0" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>archiviostorico_unibo</x:v>
+        <x:v>dl_ficlit</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Archivio Storico Universita di Bologna</x:v>
+        <x:v>FICLIT Digital Library</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
         <x:v>Italia / Emilia-Romagna</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>IIIF diretto da manifest pubblico archiviostorico.unibo.it</x:v>
+        <x:v>IIIF diretto da item Omeka S o manifest FICLIT; download da immagine diretta canvas</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
-        <x:v>Manifest pubblici consultabili; diritti e riuso da verificare a livello di singolo oggetto</x:v>
+        <x:v>Condizioni d'uso specifiche per item set/collezione; corretta citazione richiesta</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
-        <x:v>Supportare solo manifest item-level pubblici, evitare collection di annata, usare range esplicito e controllo diritti/licenza del record</x:v>
+        <x:v>Supportare solo item/manifest FICLIT pubblici, con range esplicito e verifica termini item-level; evitare tile service per HTTP 500 sui ritagli</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="198" hidden="0" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>biblioteca_digitale_trentina</x:v>
+        <x:v>archiviostorico_unibo</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Biblioteca Digitale Trentina</x:v>
+        <x:v>Archivio Storico Universita di Bologna</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>Italia / Trentino</x:v>
+        <x:v>Italia / Emilia-Romagna</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>Manifest sintetico da immagini pubbliche in pagina + PDF diretto ufficiale per testi a stampa</x:v>
+        <x:v>IIIF diretto da manifest pubblico archiviostorico.unibo.it</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>Materiali in pubblico dominio; pagina Riuso favorevole con citazione della fonte</x:v>
+        <x:v>Manifest pubblici consultabili; diritti e riuso da verificare a livello di singolo oggetto</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>Supporto tecnico su immagini pubbliche; quando l'utente richiede solo PDF e non imposta range, usare il PDF diretto ufficiale</x:v>
+        <x:v>Supportare solo manifest item-level pubblici, evitare collection di annata, usare range esplicito e controllo diritti/licenza del record</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="224.39999389648438" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>biblioteca_digitale_lombarda</x:v>
+        <x:v>phaidra_unipd</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>Biblioteca Digitale Lombarda</x:v>
+        <x:v>PHAIDRA Universita di Padova</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
-        <x:v>Italia / Lombardia</x:v>
+        <x:v>Italia / Veneto</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>Manifest sintetico da endpoint PDF REST pubblico</x:v>
+        <x:v>IIIF diretto da pagina oggetto o manifest PHAIDRA ufficiale</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
-        <x:v>Molti record dichiarano licenze non commerciale/no-derivati; diritti da verificare per item</x:v>
+        <x:v>Manifest e download pubblici presenti su alcuni oggetti; rights notice e licenza variano a livello item</x:v>
       </x:c>
       <x:c r="G12" s="10" t="str">
-        <x:v>Supportare solo documento singolo PDF da endpoint REST pubblico; niente immagini, registro o sequenze finche IIIF/info.json non risultano stabili</x:v>
+        <x:v>Supportare solo manifest item-level pubblici, con range esplicito e verifica obbligatoria di rights notice/licenza del singolo oggetto</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>rovereto_digital_library</x:v>
+        <x:v>biblioteca_digitale_trentina</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>Rovereto Digital Library</x:v>
+        <x:v>Biblioteca Digitale Trentina</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
         <x:v>Italia / Trentino</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>Manifest sintetico da API DSpace-GLAM e bitstream pagina pubblici</x:v>
+        <x:v>Manifest sintetico da immagini pubbliche in pagina + PDF diretto ufficiale per testi a stampa</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
-        <x:v>Medio</x:v>
+        <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F13" s="10" t="str">
-        <x:v>Accesso libero ai file digitali in risoluzione web secondo licenza item-level; campioni osservati CC BY-NC-ND</x:v>
+        <x:v>Materiali in pubblico dominio; pagina Riuso favorevole con citazione della fonte</x:v>
       </x:c>
       <x:c r="G13" s="10" t="str">
-        <x:v>Supportare solo bitstream classificati come pagine iiifpdf-*.png, con range esplicito per record e controllo licenza del singolo item</x:v>
+        <x:v>Supporto tecnico su immagini pubbliche; quando l'utente richiede solo PDF e non imposta range, usare il PDF diretto ufficiale</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A14" s="10" t="str">
-        <x:v>memooria</x:v>
+        <x:v>biblioteca_digitale_lombarda</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>Memooria/Jarvis</x:v>
+        <x:v>Biblioteca Digitale Lombarda</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
-        <x:v>Italia</x:v>
+        <x:v>Italia / Lombardia</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>IIIF da meta/iiif/{guid}/manifest</x:v>
+        <x:v>Manifest sintetico da endpoint PDF REST pubblico</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>Medio</x:v>
+        <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
-        <x:v>Piattaforma IIIF/API; diritti e accessi dipendono dall'ente che pubblica la collezione</x:v>
+        <x:v>Molti record dichiarano licenze non commerciale/no-derivati; diritti da verificare per item</x:v>
       </x:c>
       <x:c r="G14" s="10" t="str">
-        <x:v>Usare come capability tecnica, non come portale unico: richiedere verifica per ogni istanza</x:v>
+        <x:v>Supportare solo documento singolo PDF da endpoint REST pubblico; niente immagini, registro o sequenze finche IIIF/info.json non risultano stabili</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>vatlib</x:v>
+        <x:v>rovereto_digital_library</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>DigiVatLib</x:v>
+        <x:v>Rovereto Digital Library</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
-        <x:v>Italia / Vaticano</x:v>
+        <x:v>Italia / Trentino</x:v>
       </x:c>
       <x:c r="D15" s="10" t="str">
-        <x:v>IIIF diretto da view/mss/iiif</x:v>
+        <x:v>Manifest sintetico da API DSpace-GLAM e bitstream pagina pubblici</x:v>
       </x:c>
       <x:c r="E15" s="10" t="str">
-        <x:v>Basso-Medio</x:v>
+        <x:v>Medio</x:v>
       </x:c>
       <x:c r="F15" s="10" t="str">
-        <x:v>Solo studio/personale; riproduzione o pubblicazione richiede autorizzazione BAV</x:v>
+        <x:v>Accesso libero ai file digitali in risoluzione web secondo licenza item-level; campioni osservati CC BY-NC-ND</x:v>
       </x:c>
       <x:c r="G15" s="10" t="str">
-        <x:v>Mantenere con avviso forte e senza presentarlo come fonte liberamente riusabile</x:v>
+        <x:v>Supportare solo bitstream classificati come pagine iiifpdf-*.png, con range esplicito per record e controllo licenza del singolo item</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>findbuch</x:v>
+        <x:v>doge_unige</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
-        <x:v>Kirchenbuecher Suedtirol / findbuch.net</x:v>
+        <x:v>DOGE Digital Library / Universita di Genova</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
-        <x:v>Alto Adige / Sudtirol</x:v>
+        <x:v>Italia / Liguria</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
-        <x:v>Manifest sintetico da HTML + gtpc.php</x:v>
+        <x:v>Manifest sintetico da API DSpace-GLAM e derivati pubblici IIIF-ALTERNATIVE-*</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Medio</x:v>
       </x:c>
       <x:c r="F16" s="10" t="str">
-        <x:v>Piattaforma tecnica per molti enti; diritti/contenuti dipendono dalla singola subdomain</x:v>
+        <x:v>Fonti SBA UniGe indicano CC BY-SA per gli oggetti UniGe e CC0 per i metadati; verificare comunque la licenza del singolo item</x:v>
       </x:c>
       <x:c r="G16" s="10" t="str">
-        <x:v>Mantenere solo per risorse pubbliche e range puntuale; non estendere senza termini dell'ente</x:v>
+        <x:v>Supportare solo derivati pubblici IIIF-ALTERNATIVE-LD e PDF IIIF-ALTERNATIVE-DOWNLOAD, con range esplicito; escludere ORIGINAL e bundle IIIF-PDF-* segnati nodownload</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="132" hidden="0" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>matricula</x:v>
+        <x:v>memooria</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>Matricula Online</x:v>
+        <x:v>Memooria/Jarvis</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
-        <x:v>Europa centrale</x:v>
+        <x:v>Italia</x:v>
       </x:c>
       <x:c r="D17" s="10" t="str">
-        <x:v>Manifest sintetico da viewer HTML e hosted-images</x:v>
+        <x:v>IIIF da meta/iiif/{guid}/manifest</x:v>
       </x:c>
       <x:c r="E17" s="10" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Medio</x:v>
       </x:c>
       <x:c r="F17" s="10" t="str">
-        <x:v>Immagini registri CC BY-NC-ND 2.0; pubblicazioni e dati soggetti a obblighi/leggi locali</x:v>
+        <x:v>Piattaforma IIIF/API; diritti e accessi dipendono dall'ente che pubblica la collezione</x:v>
       </x:c>
       <x:c r="G17" s="10" t="str">
-        <x:v>Mantenere con limite non commerciale, no derivati, citazione/link e senza bulk scraping</x:v>
+        <x:v>Usare come capability tecnica, non come portale unico: richiedere verifica per ogni istanza</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>gallica</x:v>
+        <x:v>vatlib</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>Gallica (BnF)</x:v>
+        <x:v>DigiVatLib</x:v>
       </x:c>
       <x:c r="C18" s="10" t="str">
-        <x:v>Francia</x:v>
+        <x:v>Italia / Vaticano</x:v>
       </x:c>
       <x:c r="D18" s="10" t="str">
-        <x:v>IIIF diretto da ARK + fallback Playwright per TLS/fingerprint</x:v>
+        <x:v>IIIF diretto da view/mss/iiif</x:v>
       </x:c>
       <x:c r="E18" s="10" t="str">
-        <x:v>Medio</x:v>
+        <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F18" s="10" t="str">
-        <x:v>API IIIF aperta salvo abuso; riuso non commerciale libero con citazione, commerciale soggetto a licenza</x:v>
+        <x:v>Solo studio/personale; riproduzione o pubblicazione richiede autorizzazione BAV</x:v>
       </x:c>
       <x:c r="G18" s="10" t="str">
-        <x:v>Consolidare con citazione obbligatoria, rispetto del non commerciale e cautela sui partner</x:v>
+        <x:v>Mantenere con avviso forte e senza presentarlo come fonte liberamente riusabile</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="str">
-        <x:v>heidelberg</x:v>
+        <x:v>findbuch</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Heidelberg UB</x:v>
+        <x:v>Kirchenbuecher Suedtirol / findbuch.net</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>Germania</x:v>
+        <x:v>Alto Adige / Sudtirol</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
-        <x:v>IIIF diretto + rate-limit sequenziale</x:v>
+        <x:v>Manifest sintetico da HTML + gtpc.php</x:v>
       </x:c>
       <x:c r="E19" s="10" t="str">
-        <x:v>Basso-Medio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="F19" s="10" t="str">
-        <x:v>Licenza da verificare per volume: Public Domain, CC-BY-SA 4.0 o In Copyright</x:v>
+        <x:v>Piattaforma tecnica per molti enti; diritti/contenuti dipendono dalla singola subdomain</x:v>
       </x:c>
       <x:c r="G19" s="10" t="str">
-        <x:v>Consolidare con credito fonte e controllo licenza per singolo volume</x:v>
+        <x:v>Mantenere solo per risorse pubbliche e range puntuale; non estendere senza termini dell'ente</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A20" s="10" t="str">
-        <x:v>bodleian</x:v>
+        <x:v>matricula</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>Bodleian Libraries Oxford</x:v>
+        <x:v>Matricula Online</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
-        <x:v>Regno Unito</x:v>
+        <x:v>Europa centrale</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
-        <x:v>IIIF diretto da object UUID</x:v>
+        <x:v>Manifest sintetico da viewer HTML e hosted-images</x:v>
       </x:c>
       <x:c r="E20" s="10" t="str">
-        <x:v>Basso</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="F20" s="10" t="str">
-        <x:v>In prevalenza CC-BY-NC 4.0 con attribuzione; verificare restrizioni del singolo item</x:v>
+        <x:v>Immagini registri CC BY-NC-ND 2.0; pubblicazioni e dati soggetti a obblighi/leggi locali</x:v>
       </x:c>
       <x:c r="G20" s="10" t="str">
-        <x:v>Consolidare IIIF con avviso non commerciale, attribuzione e niente re-hosting sistematico immagini</x:v>
+        <x:v>Mantenere con limite non commerciale, no derivati, citazione/link e senza bulk scraping</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="132" hidden="0" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>e_rara</x:v>
+        <x:v>gallica</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>e-rara</x:v>
+        <x:v>Gallica (BnF)</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
-        <x:v>Svizzera</x:v>
+        <x:v>Francia</x:v>
       </x:c>
       <x:c r="D21" s="10" t="str">
-        <x:v>IIIF builder dedicato</x:v>
+        <x:v>IIIF diretto da ARK + fallback Playwright per TLS/fingerprint</x:v>
       </x:c>
       <x:c r="E21" s="10" t="str">
-        <x:v>Basso-Medio</x:v>
+        <x:v>Medio</x:v>
       </x:c>
       <x:c r="F21" s="10" t="str">
-        <x:v>Licenza dichiarata per documento: Public Domain Mark o CC BY-SA 4.0</x:v>
+        <x:v>API IIIF aperta salvo abuso; riuso non commerciale libero con citazione, commerciale soggetto a licenza</x:v>
       </x:c>
       <x:c r="G21" s="10" t="str">
-        <x:v>Consolidare con controllo licenza per documento e citazione della fonte</x:v>
+        <x:v>Consolidare con citazione obbligatoria, rispetto del non commerciale e cautela sui partner</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A22" s="10" t="str">
-        <x:v>e_codices</x:v>
+        <x:v>heidelberg</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>e-codices (Unifr)</x:v>
+        <x:v>Heidelberg UB</x:v>
       </x:c>
       <x:c r="C22" s="10" t="str">
-        <x:v>Svizzera</x:v>
+        <x:v>Germania</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>IIIF builder dedicato</x:v>
+        <x:v>IIIF diretto + rate-limit sequenziale</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F22" s="10" t="str">
-        <x:v>Uso non commerciale libero con citazione; eccezioni Public Domain/Creative Commons per item marcati</x:v>
+        <x:v>Licenza da verificare per volume: Public Domain, CC-BY-SA 4.0 o In Copyright</x:v>
       </x:c>
       <x:c r="G22" s="10" t="str">
-        <x:v>Consolidare con citazione obbligatoria e avviso per usi commerciali/pubblicazioni</x:v>
+        <x:v>Consolidare con credito fonte e controllo licenza per singolo volume</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A23" s="10" t="str">
-        <x:v>e_manuscripta</x:v>
+        <x:v>bodleian</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>e-manuscripta</x:v>
+        <x:v>Bodleian Libraries Oxford</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
-        <x:v>Svizzera</x:v>
+        <x:v>Regno Unito</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
-        <x:v>IIIF builder dedicato</x:v>
+        <x:v>IIIF diretto da object UUID</x:v>
       </x:c>
       <x:c r="E23" s="10" t="str">
-        <x:v>Basso-Medio</x:v>
+        <x:v>Basso</x:v>
       </x:c>
       <x:c r="F23" s="10" t="str">
-        <x:v>Licenza dichiarata per documento; alcuni contenuti hanno diritti limitati di terzi</x:v>
+        <x:v>In prevalenza CC-BY-NC 4.0 con attribuzione; verificare restrizioni del singolo item</x:v>
       </x:c>
       <x:c r="G23" s="10" t="str">
-        <x:v>Consolidare con controllo licenza per documento; evitare copia sistematica/re-hosting</x:v>
+        <x:v>Consolidare IIIF con avviso non commerciale, attribuzione e niente re-hosting sistematico immagini</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A24" s="10" t="str">
-        <x:v>internet_archive</x:v>
+        <x:v>e_rara</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>Internet Archive</x:v>
+        <x:v>e-rara</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
-        <x:v>Internazionale</x:v>
+        <x:v>Svizzera</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
-        <x:v>Manifest sintetico da metadata/files/BookReaderImages</x:v>
+        <x:v>IIIF builder dedicato</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>Medio-Alto</x:v>
+        <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
-        <x:v>Licenza e disponibilita variabili per item; alcuni item sono prestito o no-download</x:v>
+        <x:v>Licenza dichiarata per documento: Public Domain Mark o CC BY-SA 4.0</x:v>
       </x:c>
       <x:c r="G24" s="10" t="str">
-        <x:v>Supportare solo item pubblici scaricabili, con licenza/diritti chiari e senza aggirare prestito/no-download</x:v>
+        <x:v>Consolidare con controllo licenza per documento e citazione della fonte</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="132" hidden="0" customHeight="1">
       <x:c r="A25" s="10" t="str">
-        <x:v>europeana</x:v>
+        <x:v>e_codices</x:v>
       </x:c>
       <x:c r="B25" s="10" t="str">
-        <x:v>Europeana IIIF</x:v>
+        <x:v>e-codices (Unifr)</x:v>
       </x:c>
       <x:c r="C25" s="10" t="str">
-        <x:v>Internazionale</x:v>
+        <x:v>Svizzera</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>IIIF diretto da provider/record id</x:v>
+        <x:v>IIIF builder dedicato</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>Diritti da leggere per record/provider; API soggetta a chiave, termini e limiti</x:v>
+        <x:v>Uso non commerciale libero con citazione; eccezioni Public Domain/Creative Commons per item marcati</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>Usare solo record con IIIF disponibile, rights statement chiaro e attribution ai provider</x:v>
+        <x:v>Consolidare con citazione obbligatoria e avviso per usi commerciali/pubblicazioni</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A26" s="10" t="str">
+        <x:v>e_manuscripta</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>e-manuscripta</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>Svizzera</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="str">
+        <x:v>IIIF builder dedicato</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>Basso-Medio</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="str">
+        <x:v>Licenza dichiarata per documento; alcuni contenuti hanno diritti limitati di terzi</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str">
+        <x:v>Consolidare con controllo licenza per documento; evitare copia sistematica/re-hosting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>internet_archive</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Internet Archive</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Internazionale</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Manifest sintetico da metadata/files/BookReaderImages</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>Medio-Alto</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>Licenza e disponibilita variabili per item; alcuni item sono prestito o no-download</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>Supportare solo item pubblici scaricabili, con licenza/diritti chiari e senza aggirare prestito/no-download</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>europeana</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Europeana IIIF</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Internazionale</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>IIIF diretto da provider/record id</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Basso-Medio</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Diritti da leggere per record/provider; API soggetta a chiave, termini e limiti</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>Usare solo record con IIIF disponibile, rights statement chiaro e attribution ai provider</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
         <x:v>manifest_diretto</x:v>
       </x:c>
-      <x:c r="B26" s="10" t="str">
+      <x:c r="B29" t="str">
         <x:v>Manifest diretto (URL gia noto)</x:v>
       </x:c>
-      <x:c r="C26" s="10" t="str">
+      <x:c r="C29" t="str">
         <x:v>Avanzato</x:v>
       </x:c>
-      <x:c r="D26" s="10" t="str">
+      <x:c r="D29" t="str">
         <x:v>URL manifest fornito dall'utente</x:v>
       </x:c>
-      <x:c r="E26" s="10" t="str">
+      <x:c r="E29" t="str">
         <x:v>Variabile</x:v>
       </x:c>
-      <x:c r="F26" s="10" t="str">
+      <x:c r="F29" t="str">
         <x:v>Responsabilita utente + verifica termini origine</x:v>
       </x:c>
-      <x:c r="G26" s="10" t="str">
+      <x:c r="G29" t="str">
         <x:v>Mantenere con avviso/criteri chiari</x:v>
       </x:c>
     </x:row>
@@ -958,16 +1027,16 @@
         <x:v>Italia</x:v>
       </x:c>
       <x:c r="D2" s="10" t="str">
-        <x:v>https://icar.cultura.gov.it/sistemi-e-portali/archivi-nazionali; https://archivinazionali.cultura.gov.it/; https://icar.cultura.gov.it/sistemi-e-portali/archivi-nazionali/sala-studio</x:v>
+        <x:v>https://icar.cultura.gov.it/sistemi-e-portali/archivi-nazionali; https://archivinazionali.cultura.gov.it/; https://icar.cultura.gov.it/sistemi-e-portali/archivi-nazionali/sala-studio; https://icar.cultura.gov.it/sistemi-e-portali/archivi-nazionali/sia</x:v>
       </x:c>
       <x:c r="E2" s="10" t="str">
         <x:v>Molto alta: ricerca trasversale su fondi archivistici, Antenati, Archivi di Stato, Soprintendenze e progetti di digitalizzazione</x:v>
       </x:c>
       <x:c r="F2" s="10" t="str">
-        <x:v>Controllo 2026-06-05: il nuovo portale Archivi Nazionali risulta ancora in sviluppo; la pagina ICAR prevede accesso gratuito ma anche risorse fruibili solo previa identita digitale; Sala Studio richiede SPID/CIE/eIDAS per richieste e riproduzioni</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: ICAR conferma che il nuovo SIA e' il contesto unificato destinato a integrare SIAS, SIUSA, Strumenti di ricerca online e Archivio Digitale nella futura architettura Archivi Nazionali. Sala Studio e' ora un servizio operativo, accessibile solo con SPID/CIE/eIDAS, per consultazione in sede, richieste di riproduzione, ricerche da remoto e consulenze; la notizia ufficiale del 2026-06-30 conferma 64 Archivi di Stato attivi dal 1 luglio 2026. Il quadro rafforza la rilevanza strategica del portale, ma non fa emergere una capability downloader pubblica no-login</x:v>
       </x:c>
       <x:c r="G2" s="10" t="str">
-        <x:v>C - candidato strategico solo per discovery/link assistito; nessun downloader finche il portale non e pubblico, stabile e dotato di API/IIIF e termini compatibili</x:v>
+        <x:v>C - candidato strategico per discovery/link assistito e accesso ai servizi; nessun downloader finche non emergono API/IIIF/endpoint pubblici compatibili</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="488.3999938964844" hidden="0" customHeight="1">
@@ -981,16 +1050,16 @@
         <x:v>Italia</x:v>
       </x:c>
       <x:c r="D3" s="10" t="str">
-        <x:v>https://archiviodigitale-icar.cultura.gov.it/; https://archiviodigitale-icar.cultura.gov.it/it/172/termini-d-uso; https://archiviodigitale-icar.cultura.gov.it/it/163/guida-alla-ricerca</x:v>
+        <x:v>https://archiviodigitale-icar.cultura.gov.it/; https://archiviodigitale-icar.cultura.gov.it/it/172/termini-d-uso; https://archiviodigitale-icar.cultura.gov.it/it/163/guida-alla-ricerca; pagina ICAR https://icar.cultura.gov.it/sistemi-e-portali/sistemi-legacy/archivio-digitale</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
         <x:v>Molto alta: 46 istituti sul portale, progetti di digitalizzazione, fondi, complessi e unita documentarie; contiene anche fonti genealogiche e archivistiche molto rilevanti</x:v>
       </x:c>
       <x:c r="F3" s="10" t="str">
-        <x:v>Consultazione gratuita e no-login; termini d'uso CC BY-NC-SA dove non diversamente specificato, ma divieto espresso di copia/estrazione massiva, robot o metodi analoghi, reverse engineering e aggiramento sicurezza. Tecnicamente utile come portale di ricerca, ma non compatibile con downloader ATK-Pro</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: Archivio Digitale resta pubblico, gratuito e consultabile senza registrazione, con 46 istituti presenti e ricerca su progetti, fondi, complessi e unita' documentarie. La pagina ICAR aggiornata al 2026-05-15 lo conferma come strumento centrale di consultazione del patrimonio digitalizzato. I termini d'uso continuano pero' a vietare copia/estrazione massiva, robot o metodi analoghi, reverse engineering e aggiramento delle misure di sicurezza</x:v>
       </x:c>
       <x:c r="G3" s="10" t="str">
-        <x:v>C - link/discovery assistito; vietare builder/downloader e live smoke di download, salvo futuro endpoint ufficiale documentato e autorizzato</x:v>
+        <x:v>C - link/discovery assistito e consultazione pubblica; vietare builder/downloader e live smoke di download salvo futuro endpoint ufficiale documentato e autorizzato</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="528" hidden="0" customHeight="1">
@@ -1010,10 +1079,10 @@
         <x:v>Alta: descrizioni di Archivi di Stato, inventari, strumenti di ricerca e possibili riproduzioni digitali collegate a schede</x:v>
       </x:c>
       <x:c r="F4" s="10" t="str">
-        <x:v>Controllo 2026-06-05: DGA/ICAR descrivono SIAS come sistema descrittivo; gli strumenti di ricerca online rimandano a inventari pubblicati nel web o nel portale SAN, in formato dinamico o PDF. ICAR segnala riproduzioni digitali collegate tramite metadati MAG-SIAS, ma non emerge una API/IIIF o policy downloader generale</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-29: DGA continua a descrivere SIAS come sistema di descrizione del patrimonio documentario degli Archivi di Stato, con accesso agli strumenti di ricerca pubblicati online quando esistono. Il ricontrollo conferma il ruolo descrittivo/inventariale e non fa emergere una capability downloader autonoma; inoltre il quadro ICAR 2026 colloca SIAS nel percorso di integrazione verso il nuovo SIA</x:v>
       </x:c>
       <x:c r="G4" s="10" t="str">
-        <x:v>C - link/discovery e apertura inventari; no download immagini o PDF massivo senza endpoint e termini specifici</x:v>
+        <x:v>C - discovery/link assistito e apertura inventari; no download immagini o PDF massivo senza endpoint e termini specifici</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="475.20001220703125" hidden="0" customHeight="1">
@@ -1033,10 +1102,10 @@
         <x:v>Alta: punto di accesso unificato a risorse archivistiche nazionali, catalogo CAT, inventari e risorse digitali collegate</x:v>
       </x:c>
       <x:c r="F5" s="10" t="str">
-        <x:v>Controllo 2026-06-05: DGA presenta SAN come catalogo/interoperabilita e accesso a fondi o serie consultabili digitalmente presso sistemi aderenti; Strumenti di ricerca online e orientato a inventari e descrizioni. Esiste una pista OAI/open data per metadati, ma immagini e diritti restano del sistema sorgente</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-29: DGA continua a presentare SAN come catalogo/interoperabilita e accesso a fondi o serie consultabili digitalmente presso sistemi aderenti; Strumenti di ricerca online resta orientato a inventari e descrizioni. L'endpoint ufficiale oaicat continua a documentare un OAI Provider open data con set SAN e baseURL http://www.san.beniculturali.it/oaicat/OAIHandler, quindi la pista metadata/OAI e' reale e stabile. Resta pero' una capability di metadati: immagini, PDF e diritti dipendono dai sistemi sorgente</x:v>
       </x:c>
       <x:c r="G5" s="10" t="str">
-        <x:v>B/C - possibile futura capability metadata/OAI se stabile e documentata; no downloader immagini diretto</x:v>
+        <x:v>B - capability futura metadata/OAI piu' concreta; no downloader immagini diretto via SAN</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="462" hidden="0" customHeight="1">
@@ -1050,13 +1119,13 @@
         <x:v>Italia</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>https://archivi.cultura.gov.it/strumenti-di-ricerca-online/il-sistema-informativo-unificato-per-le-soprintendenze-archivistiche-siusa; https://siusa-archivi.cultura.gov.it/cgi-bin/siusa/pagina.pl?TipoPag=informazioni; https://siusa-archivi.cultura.gov.it/cgi-bin/siusa/pagina.pl?RicVM=inventari</x:v>
+        <x:v>https://archivi.cultura.gov.it/strumenti-di-ricerca-online/il-sistema-informativo-unificato-per-le-soprintendenze-archivistiche-siusa; https://siusa-archivi.cultura.gov.it/cgi-bin/siusa/pagina.pl?TipoPag=informazioni; https://siusa-archivi.cultura.gov.it/cgi-bin/siusa/pagina.pl?RicVM=inventari; riferimento ICAR 2026 https://icar.cultura.gov.it/sistemi-e-portali/sistemi-nazionali-di-descrizione-archivistica/sistema-informativo-unificato-per-le-soprintendenze-archivistiche-siusa-1</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
         <x:v>Media-alta: censimento archivi pubblici e privati vigilati, soggetti conservatori/produttori, inventari e percorsi regionali/tematici</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
-        <x:v>Controllo 2026-06-05: SIUSA e punto di accesso primario per patrimonio archivistico non statale; consente accesso a inventari online interni o esterni e dal 2011 esporta dati nel SAN. Il sito indica licenza CC BY-SA per i testi salvo diversa specificazione, ma non e un portale immagini/downloader</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-29: SIUSA continua a presentarsi come banca dati di complessi archivistici, soggetti e strumenti di ricerca, con inventari online interni o esterni al sistema. Il ruolo utile per ATK-Pro resta discovery/contesto; non emerge una capability downloader immagini autonoma. Anche SIUSA rientra nel percorso ICAR di integrazione verso il nuovo SIA</x:v>
       </x:c>
       <x:c r="G6" s="10" t="str">
         <x:v>C - discovery, schede e link assistito; eventuale metadata solo via SAN/open data, nessun downloader</x:v>
@@ -1079,10 +1148,10 @@
         <x:v>Molto alta per genealogia preunitaria e ricerca ecclesiastica: censimento di beni archivistici, istituti culturali, soggetti conservatori, persone, famiglie, enti e inventari ecclesiastici</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>Controllo 2026-06-05: BeWeB e la vetrina nazionale del censimento CEI; CEI-Ar pubblica banche dati/inventari di archivi ecclesiastici e puo collegare immagini a schede. I termini indicano CC BY-NC-SA per i contenuti, CC0 solo per dati catalografici di Persone, Famiglie e Istituti culturali; esistono area riservata e servizi di prenotazione. Non emerge una API/IIIF pubblica generalizzabile o una policy di download immagini</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: BeWeB continua a presentarsi come vetrina nazionale del censimento CEI con ricerca trasversale e pubblicazione progressiva degli inventari prodotti nella rete CEI-Ar. La pubblicazione online avviene tramite accordi e liberatorie degli istituti aderenti. I termini restano differenziati: CC0 per Persone, Famiglie e Istituti culturali; CC BY-NC-SA per gli altri contenuti, con possibili diritti di terzi. Su alcune schede pubbliche compaiono anche indicazioni item-level di licenza e il comando di copia del manifest IIIF, ma non emerge una capability uniforme e generalizzabile per download automatico</x:v>
       </x:c>
       <x:c r="G7" s="10" t="str">
-        <x:v>C - discovery/link assistito e, al massimo, futura metadata/search su dati catalografici compatibili; no downloader</x:v>
+        <x:v>C - discovery/link assistito e, al massimo, futura metadata/search su dati catalografici compatibili; no downloader generico</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="541.2000122070312" hidden="0" customHeight="1">
@@ -1096,13 +1165,13 @@
         <x:v>Italia ecclesiastica</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>https://www.beweb.chiesacattolica.it/beniarchivistici/aggregatore/3/Dove%2B-%2BI%2BSoggetti%2BConservatori%2B%3A%2BArchivio%2Bparrocchiale; portali diocesani specifici da verificare caso per caso</x:v>
+        <x:v>https://www.beweb.chiesacattolica.it/beniarchivistici/aggregatore/3/Dove%2B-%2BI%2BSoggetti%2BConservatori%2B%3A%2BArchivio%2Bparrocchiale; https://www.beweb.chiesacattolica.it/beniarchivistici/aggregatore/1/Archivio%2Bdiocesano; portali diocesani specifici da verificare caso per caso</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
         <x:v>Molto alta: registri di battesimo, matrimonio, defunti, stati delle anime, processetti matrimoniali e archivi parrocchiali non sempre coperti da Antenati</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
-        <x:v>BeWeB conferma che gli archivi parrocchiali rientrano tra i soggetti conservatori e collega categorie genealogiche esplicite; tuttavia accesso, riproduzione, privacy, conservazione fisica e digitalizzazione dipendono dalla diocesi/parrocchia. Molte fonti possono richiedere contatto, appuntamento, autorizzazione o consultazione locale</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: BeWeB continua a confermare che gli archivi parrocchiali e diocesani custodiscono le serie genealogicamente piu' rilevanti e che il luogo di conservazione/consultazione puo' variare caso per caso. Le notizie BeWeB 2026 confermano inoltre una crescita della pubblicazione di fondi archivistici e, quando l'istituto aderente lo consente, la possibilita' di esplorare fino alle singole unita' archivistiche. Questo rafforza la funzione di scouting/orientamento, ma accesso, riproduzione, privacy e digitalizzazione restano dipendenti dalla diocesi/parrocchia o dall'archivio storico competente</x:v>
       </x:c>
       <x:c r="G8" s="10" t="str">
         <x:v>C - mappa/link assistiti e schede di orientamento; vietare automazioni generiche, login, aree riservate e download senza fonte pubblica no-login con termini chiari</x:v>
@@ -1119,13 +1188,13 @@
         <x:v>Svizzera italiana</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>https://www4.ti.ch/decs/dcsu/asti/servizi/servizio-archivi-locali-sal/; https://www4.ti.ch/fileadmin/DECS/DCSU/ASTI/Documenti/Ricerche_genealogiche.pdf</x:v>
+        <x:v>https://www4.ti.ch/decs/dcsu/asti/servizi/servizio-archivi-locali-sal/; https://www4.ti.ch/fileadmin/DECS/DCSU/ASTI/Documenti/Ricerche_genealogiche.pdf; https://www4.ti.ch/decs/dcsu/asti/servizi/consultazione-e-riproduzione-dei-documenti/; catalogo https://www.archiviodistato.ti.ch/Query/volltextsuche.aspx</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>Molto alta per Ticino: fondi genealogici 1750-1960, archivi comunali, patriziali e parrocchiali, ruoli di popolazione, stato civile e microfilm ecclesiastici</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>Controllo 2026-06-05: ASTi/SAL censisce e riordina oltre 600 archivi locali, compresi archivi parrocchiali. Le disposizioni genealogiche indicano ricerche puntuali, formulari, costi dopo i primi 30 minuti, restrizioni su ruoli di popolazione/passaporti e divieto di riproduzione sistematica dei Ruoli di Popolazione. I registri parrocchiali ticinesi risultano disponibili online via FamilySearch e su microfilm presso Archivio diocesano di Lugano, non come endpoint pubblico ASTi</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: ASTi/SAL continua a censire e riordinare archivi locali, compresi archivi parrocchiali, e offre strumenti online reali come il catalogo scopeArchiv. La consultazione in sede o in versione digitale resta gratuita, ma regolamento e tariffario confermano emolumenti per alcuni servizi, comprese riproduzioni digitali e supporti di ricerca approfonditi. Le ricerche genealogiche restano soggette a condizioni particolari e a richieste puntuali via formulario; i registri parrocchiali ticinesi risultano ancora accessibili soprattutto tramite FamilySearch o microfilm presso l'Archivio diocesano di Lugano, non come endpoint pubblico ASTi</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
         <x:v>C - link/manuale e schede di orientamento; no downloader ATK-Pro</x:v>
@@ -1142,13 +1211,13 @@
         <x:v>Svizzera italiana ecclesiastica</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>https://www.diocesilugano.ch/uffici-della-curia/; https://www4.ti.ch/decs/dcsu/uapcd/osservatorio/banca-dati-operatori-culturali/dettaglio/?tx_tichosservatorio_decsocoperatori%5Bid%5D=294</x:v>
+        <x:v>https://www.diocesilugano.ch/uffici-della-curia/; https://www4.ti.ch/decs/dcsu/uapcd/osservatorio/banca-dati-operatori-culturali/dettaglio/?tx_tichosservatorio_decsocoperatori%5Bid%5D=294; avvisi https://www.diocesilugano.ch/category/news/</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
         <x:v>Alta: microfilm e consultazione ecclesiastica per registri parrocchiali ticinesi, utile per fonti precedenti o complementari allo stato civile</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
-        <x:v>La diocesi indica consultazione dell'Archivio storico su appuntamento; le disposizioni ASTi citano copie microfilm dei registri parrocchiali presso l'Archivio diocesano di Lugano. Non emerge portale pubblico con immagini scaricabili o API</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: la diocesi continua a indicare l'Archivio storico come servizio di consultazione su appuntamento nei giorni feriali, salvo il mercoledi, e pubblica anche avvisi operativi come la chiusura estiva 2026 con riapertura il 18 agosto. Le disposizioni ASTi citano copie microfilm dei registri parrocchiali presso l'Archivio diocesano di Lugano. Non emerge comunque un portale pubblico con immagini scaricabili o API</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
         <x:v>C - solo contatto/link assistito e istruzioni di consultazione</x:v>
@@ -1165,16 +1234,16 @@
         <x:v>Grigioni italofoni / area retica</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/familienforschung/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/Seiten/default.aspx</x:v>
+        <x:v>https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/familienforschung/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/chisiamo/Seiten/default.aspx</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>Molto alta per valli italofone, mobilita alpina e fonti pre-1876: registri parrocchiali, stato civile, registri dei cittadini, schede genealogiche e strumenti di ricerca</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>Controllo 2026-06-05: l'Archivio di Stato indica microfilm di tutti i registri parrocchiali conosciuti, consultabili presso l'Archivio; registri di stato civile fino al 1929 in sala lettura; registri delle famiglie non visionabili; alcuni registri dei cittadini soggetti ad autorizzazione. Il sistema informativo e i PDF sono online, ma i documenti d'archivio sono in gran parte non accessibili online e vanno consultati in sala lettura</x:v>
+        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: l'Archivio di Stato conferma che tutti i registri parrocchiali noti sono stati microfilmati e consultabili presso l'Archivio; i registri di stato civile fino al 1929 sono consultabili in sala di lettura, quelli dei cittadini attinenti fino al 1929 su microfilm, mentre i registri delle famiglie dal 1929 non sono visionabili. Il quadro online e' piu' ricco di quanto sembrasse: oltre a PDF e sistema informativo, il sito indica fondi digitalizzati consultabili online e integrazione con Archives Online per metadati e documenti delle banche dati collegate. Resta comunque un ramo soprattutto consultativo e regolato</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>C - discovery/link assistito; no download, salvo eventuali fondi digitalizzati con condizioni specifiche</x:v>
+        <x:v>C - discovery/link assistito; no download generale, salvo eventuali fondi digitalizzati con condizioni specifiche</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="435.6000061035156" hidden="0" customHeight="1">
@@ -1188,13 +1257,13 @@
         <x:v>Grigioni / area retica ecclesiastica</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>https://www.archiv-bistum-chur.ch/; https://www.bistumsarchiv-chur.findbuch.net/</x:v>
+        <x:v>https://www.archiv-bistum-chur.ch/; https://www.bistumsarchiv-chur.findbuch.net/; contatti https://www.archiv-bistum-chur.ch/Kontakt.htm</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
         <x:v>Alta: diocesi storica antica, rilevante per fonti ecclesiastiche grigionesi e area retica</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
-        <x:v>Il sito ufficiale documenta l'ordinamento, indicizzazione e apertura digitale del patrimonio storico e moderno e rimanda a un sistema Findbuch; non emerge una policy di download immagini/API generalizzabile. Da trattare come ricerca guidata e link a inventari</x:v>
+        <x:v>Ricontrollo ufficiale 2026-07-31: il sito documenta un archivio ecclesiastico strutturato, con ordinamento dei fondi, repertori online, Findbuch e lavori di digitalizzazione/descrizione in corso su varie serie. La pagina contatti esplicita pero' che il BAC non e' un archivio pubblico: la consultazione e' solo previa richiesta, nel locale di lettura/lavoro e secondo un regolamento proprio. Non emerge quindi una policy di download immagini/API generalizzabile</x:v>
       </x:c>
       <x:c r="G12" s="10" t="str">
         <x:v>C - link/discovery assistito; non estendere come downloader generico</x:v>
@@ -1263,7 +1332,7 @@
         <x:v>Alta per libri antichi, manoscritti, periodici, editoria lombarda e fonti bibliografiche utili alla ricerca genealogica e territoriale</x:v>
       </x:c>
       <x:c r="F15" s="10" t="str">
-        <x:v>Controllo 2026-06-08: termini ufficiali molto favorevoli per opere in pubblico dominio, immagini scaricabili/riutilizzabili e dati CC0; infrastruttura Rosetta/Alma/Primo VE con OAI-PMH documentato. Lato download non e ancora emerso un endpoint utilizzabile in modo ripetibile: il test live su Preserver IE7400509 ha trovato solo il logo del viewer, mentre il record Primo alma9925210904741 non ha esposto candidati manifest, PDF o immagini utili alla sonda. verify_beic_technical_probe.py resta lo strumento di raccolta campioni, ma senza integrazione nel menu</x:v>
+        <x:v>Controllo 2026-06-08 + ricontrollo 2026-07-29: termini ufficiali molto favorevoli per opere in pubblico dominio, immagini scaricabili/riutilizzabili e dati CC0; infrastruttura Rosetta/Alma/Primo VE con OAI-PMH documentato. Lato download non e ancora emerso un endpoint utilizzabile in modo ripetibile: il test live su Preserver IE7400509 continua a mostrare solo viewer e logo del sito, mentre il record Primo alma9925210904741 non espone manifest, PDF o immagini utili alla sonda. Il probe ora separa esplicitamente gli asset grafici di sito dai segnali tecnici riusabili e classifica entrambi i campioni come GO/NO-GO: HOLD. verify_beic_technical_probe.py resta lo strumento di raccolta campioni, ma senza integrazione nel menu</x:v>
       </x:c>
       <x:c r="G15" s="10" t="str">
         <x:v>B/C - candidato forte per metadata e valore culturale, ma downloader sospeso finche non emergono campioni BEIC diretti con endpoint file/manifest stabile e policy item-level</x:v>
@@ -1386,369 +1455,415 @@
     </x:row>
     <x:row r="21" ht="1320" hidden="0" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>orientales_unior</x:v>
+        <x:v>impronte_digitali_unifi</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>OrienTales / Biblioteca digitale Universita di Napoli L'Orientale</x:v>
+        <x:v>Impronte Digitali / Universita di Firenze</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
-        <x:v>Italia / Campania</x:v>
+        <x:v>Italia / Toscana</x:v>
       </x:c>
       <x:c r="D21" s="10" t="str">
-        <x:v>https://www.unior.it/it/biblioteche/servizi-gli-utenti/biblioteca-digitale</x:v>
+        <x:v>https://improntedigitali.unifi.it/; news ufficiale https://www.sba.unifi.it/n2411.html; collezioni digitalizzate https://www.sba.unifi.it/p1308.html; campione https://improntedigitali.unifi.it/items/ea8510d3-4f09-41b6-b69a-5c4ff3d0d082; sonda verify_unifi_technical_probe.py</x:v>
       </x:c>
       <x:c r="E21" s="10" t="str">
-        <x:v>Media-alta: libri antichi, manoscritti in lingue orientali, materiale d'archivio, documentario, periodici, collane, carte geografiche e atlanti, con valore culturale e storico per ricerche italiane</x:v>
+        <x:v>Media-alta: periodici, fondi archivistici, materiali rari e di pregio delle biblioteche Unifi, con interesse per contesto storico toscano e universitario</x:v>
       </x:c>
       <x:c r="F21" s="10" t="str">
-        <x:v>Controllo 2026-06-08/10: fonte ufficiale indica licenze Creative Commons, framework IIIF, uso di Mirador, download laddove la licenza lo permetta, OCR e scarico metadati; la descrizione tecnica cita DSpace, mentre restano possibili tracce Omeka dai progetti precedenti. verify_orientales_technical_probe.py ora cerca sia pattern DSpace (entities, REST item, bundle, bitstream, handle e link JSON/HAL), sia record Omeka, viewer Mirador, manifest IIIF, info.json, immagini, OCR/testi e metadati candidati. Verifica manuale 2026-06-10: le pagine record finora viste mostrano "Il record non puo essere mostrato agli utenti ospiti" e contenuti riservati agli utenti affiliati; manca quindi il requisito minimo di accesso pubblico senza autenticazione. Il download non e generalizzabile senza record pubblici e licenza dell'oggetto</x:v>
+        <x:v>Controllo 2026-07-26 + ricontrollo 2026-07-29: la fonte ufficiale UniFI descrive il portale come digital library pubblica basata su DSpace-GLAM con viewer Mirador e standard IIIF. Verifica live sull'item Ricordi di architettura (ea8510d3-4f09-41b6-b69a-5c4ff3d0d082): API pubblica server/api/core/items/{uuid} leggibile senza login; bundle pubblici ORIGINAL, LICENSE e MAG; metadati item-level con dc.rights.holder UniFI e dc.rights.license = CC BY-NC-SA; file MAG scaricabile con codice 200; thumbnail generato (THUMBNAIL) accessibile come immagine JPEG pubblica, anche via endpoint item-level /thumbnail. Il ricontrollo del 2026-07-29 amplia il quadro del backend pubblico (record, entity correlate, item API, bundle, bitstream e surrogate, 410 candidati classificati), ma non cambia la sostanza: il primo bitstream immagine del bundle ORIGINAL resta 401 sul content diretto, i metadati del bitstream segnalano bitstream.viewer.provider = iiif insieme a nodownload, e non emergono manifest IIIF pubblici espliciti o info.json riusabili</x:v>
       </x:c>
       <x:c r="G21" s="10" t="str">
-        <x:v>C - sospeso/escluso dal download automatico finche non emergono record pubblici consultabili da ospite con licenza visibile e endpoint manifest/bitstream senza autenticazione</x:v>
+        <x:v>B - candidato forte e reale per backend DSpace-GLAM/IIIF, confermato in REVIEW: metadata e surrogate web pubblici si', ma senza download/manifest diretto ancora riusabile</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A22" s="10" t="str">
-        <x:v>museu_imigracao_sp</x:v>
+        <x:v>doge_unige</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>Museu da Imigracao do Estado de Sao Paulo - Acervo Digital</x:v>
+        <x:v>DOGE Digital Library / Universita di Genova</x:v>
       </x:c>
       <x:c r="C22" s="10" t="str">
-        <x:v>Brasile / diaspora italiana</x:v>
+        <x:v>Italia / Liguria</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>https://museudaimigracao.org.br/acervo/sobre-acervo; https://www.museudaimigracao.org.br/acervo/passageiros; https://museudaimigracao.org.br/acervo-e-pesquisa/acervo</x:v>
+        <x:v>https://doge.unige.net/; fonti SBA https://biblioteche.unige.it/doge_informazioni_generali, https://biblioteche.unige.it/doge_servizi_offerti; campione https://doge.unige.net/entities/publication/b1c2be2c-e1ae-4676-93e3-07e8e8398f72; sonda verify_doge_technical_probe.py</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str">
-        <x:v>Molto alta per immigrati italiani in Brasile/Sao Paulo</x:v>
+        <x:v>Media-alta: libri antichi, materiali scientifici, disegni, fondi storici e patrimonio universitario ligure, utile per contesto storico territoriale e bibliografico</x:v>
       </x:c>
       <x:c r="F22" s="10" t="str">
-        <x:v>Acervo digitale pubblico con piu di 250 mila immagini, registri di matricola, liste di bordo, carte di chiamata, richieste SACOP, iconografie, cartografie e giornali; le fonti ufficiali indicano uso/download non commerciale, ma il percorso tecnico appare basato su ricerca web e PDF/immagini pubbliche, non su IIIF/API documentata</x:v>
+        <x:v>Controllo 2026-07-26/27: le fonti ufficiali SBA descrivono DOGE come digital library basata su DSpace-GLAM, con Mirador, protocollo IIIF, OAI-PMH e licenza generale CC BY-SA per gli oggetti UniGe, CC0 per i metadati. Verifica live sul campione Euler b1c2be2c-e1ae-4676-93e3-07e8e8398f72: item API pubblico, handle persistente, dc.rights.license = CC BY-SA; bundle ORIGINAL, THUMBNAIL, BRANDED_PREVIEW, IIIF-PDF-*, IIIF-ALTERNATIVE-LD e IIIF-ALTERNATIVE-DOWNLOAD. I contenuti ORIGINAL e IIIF-PDF-* restano bloccati o marcati nodownload, ma i derivati IIIF-ALTERNATIVE-LD risultano pubblici pagina-per-pagina con 373 bitstream JPEG numerati e IIIF-ALTERNATIVE-DOWNLOAD espone un PDF derivato pubblico con codice 200. ATK-Pro ora costruisce quindi un manifest sintetico prudente solo dai derivati IIIF-ALTERNATIVE-LD, con PDF derivato in seeAlso, referer DOGE, range esplicito e senza toccare originali o frame viewer nodownload</x:v>
       </x:c>
       <x:c r="G22" s="10" t="str">
-        <x:v>B - candidato forte, ma non integrare finche non viene validata una capability pdf_direct/download diretto pubblica e testabile</x:v>
+        <x:v>A - promosso a supporto tecnico prudente R_LIMITED: solo derivati pubblici IIIF-ALTERNATIVE-LD + IIIF-ALTERNATIVE-DOWNLOAD, con controllo licenza item-level e divieto di estensione agli originali</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A23" s="10" t="str">
-        <x:v>apesp_digitalizados</x:v>
+        <x:v>orientales_unior</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>Arquivo Publico do Estado de Sao Paulo - Acervo digitalizado</x:v>
+        <x:v>OrienTales / Biblioteca digitale Universita di Napoli L'Orientale</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
-        <x:v>Brasile / diaspora italiana</x:v>
+        <x:v>Italia / Campania</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
-        <x:v>https://web.arquivoestado.sp.gov.br/web/acervo/digitalizados; https://www.arquivoestado.sp.gov.br/web/digitalizado/textual/nucleos_coloniais; https://web.arquivoestado.sp.gov.br/web/acervo/atendimento/reproducao_documentos; https://web.arquivoestado.sp.gov.br/web/acervo/solicitacao_certidoes/imigracao</x:v>
+        <x:v>https://www.unior.it/it/biblioteche/servizi-gli-utenti/biblioteca-digitale</x:v>
       </x:c>
       <x:c r="E23" s="10" t="str">
-        <x:v>Molto alta: Hospedaria, Porto di Santos, nuclei coloniali, documenti di immigrazione e colonizzazione</x:v>
+        <x:v>Media-alta: libri antichi, manoscritti in lingue orientali, materiale d'archivio, documentario, periodici, collane, carte geografiche e atlanti, con valore culturale e storico per ricerche italiane</x:v>
       </x:c>
       <x:c r="F23" s="10" t="str">
-        <x:v>Fonte ufficiale molto rilevante, ma l'acervo digitalizzato rimanda a registrazione/login e la pagina dei nuclei coloniali contiene avviso di servizio con login; la riproduzione e soggetta a credito, termini di responsabilita e valutazioni su diritto/autorizzazione. Nessun endpoint no-login/API/IIIF stabile verificato nel primo controllo</x:v>
+        <x:v>Controllo 2026-06-08/10: fonte ufficiale indica licenze Creative Commons, framework IIIF, uso di Mirador, download laddove la licenza lo permetta, OCR e scarico metadati; la descrizione tecnica cita DSpace, mentre restano possibili tracce Omeka dai progetti precedenti. verify_orientales_technical_probe.py ora cerca sia pattern DSpace (entities, REST item, bundle, bitstream, handle e link JSON/HAL), sia record Omeka, viewer Mirador, manifest IIIF, info.json, immagini, OCR/testi e metadati candidati. Verifica manuale 2026-06-10: le pagine record finora viste mostrano "Il record non puo essere mostrato agli utenti ospiti" e contenuti riservati agli utenti affiliati; manca quindi il requisito minimo di accesso pubblico senza autenticazione. Il download non e generalizzabile senza record pubblici e licenza dell'oggetto</x:v>
       </x:c>
       <x:c r="G23" s="10" t="str">
-        <x:v>C - link/manuale e discovery; download diretto escluso finche non emerge una risorsa pubblica no-login con licenza e tecnica stabili</x:v>
+        <x:v>C - sospeso/escluso dal download automatico finche non emergono record pubblici consultabili da ospite con licenza visibile e endpoint manifest/bitstream senza autenticazione</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="660" hidden="0" customHeight="1">
       <x:c r="A24" s="10" t="str">
-        <x:v>arquivo_nacional_br_sian</x:v>
+        <x:v>museu_imigracao_sp</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>Arquivo Nacional do Brasil / SIAN</x:v>
+        <x:v>Museu da Imigracao do Estado de Sao Paulo - Acervo Digital</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
         <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
-        <x:v>https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/a-imigracao-italiana-e-o-acervo-do-an; https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/quer-pesquisar-no-arquivo-nacional-acesse-o-sian; https://www.gov.br/arquivonacional/pt-br/servicos/acervos/copy_of_acervos-mais-consultados/entrada-de-estrangeiros; https://www.gov.br/arquivonacional/pt-br/servicos/bases-de-dados/bases</x:v>
+        <x:v>https://museudaimigracao.org.br/acervo/sobre-acervo; https://www.museudaimigracao.org.br/acervo/passageiros; https://museudaimigracao.org.br/acervo-e-pesquisa/acervo</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>Alta: ingresso di stranieri, vapori, acervo nazionale, Porto di Rio de Janeiro e Porto di Santos</x:v>
+        <x:v>Molto alta per immigrati italiani in Brasile/Sao Paulo</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
-        <x:v>SIAN e molto rilevante e offre documenti digitalizzati senza costo, ma le fonti ufficiali richiedono cadastro/login; la pagina SIAN espone anche controllo anti-spam/umano. La base separata Entrada de Estrangeiros - Porto do Rio de Janeiro e utile come ricerca nominale/dichiarazione, ma non e ancora un endpoint immagini/API verificato</x:v>
+        <x:v>Acervo digitale pubblico con piu di 250 mila immagini, registri di matricola, liste di bordo, carte di chiamata, richieste SACOP, iconografie, cartografie e giornali; le fonti ufficiali indicano uso/download non commerciale, ma il percorso tecnico appare basato su ricerca web e PDF/immagini pubbliche, non su IIIF/API documentata</x:v>
       </x:c>
       <x:c r="G24" s="10" t="str">
-        <x:v>C - link/manuale e discovery; non integrare download diretto SIAN per login/challenge. Rivalutare separatamente la base Rio solo se emerge un accesso pubblico documentato e testabile</x:v>
+        <x:v>B - candidato forte, ma non integrare finche non viene validata una capability pdf_direct/download diretto pubblica e testabile</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="633.5999755859375" hidden="0" customHeight="1">
       <x:c r="A25" s="10" t="str">
-        <x:v>agn_argentina_inmigrantes</x:v>
+        <x:v>apesp_digitalizados</x:v>
       </x:c>
       <x:c r="B25" s="10" t="str">
-        <x:v>Archivo General de la Nacion Argentina - buscador inmigrantes</x:v>
+        <x:v>Arquivo Publico do Estado de Sao Paulo - Acervo digitalizado</x:v>
       </x:c>
       <x:c r="C25" s="10" t="str">
-        <x:v>Argentina / diaspora italiana</x:v>
+        <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion; https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion/consulta-de-antecedentes-migratorios; https://www.argentina.gob.ar/noticias/el-archivo-general-de-la-nacion-es-memoria-del-mundo; https://www.argentina.gob.ar/terminos-y-condiciones; https://www.unesco.org/es/memory-world/lac/passengers-entry-books-sea-1882-1937-national-registry-migrations-documentary-fond</x:v>
+        <x:v>https://web.arquivoestado.sp.gov.br/web/acervo/digitalizados; https://www.arquivoestado.sp.gov.br/web/digitalizado/textual/nucleos_coloniais; https://web.arquivoestado.sp.gov.br/web/acervo/atendimento/reproducao_documentos; https://web.arquivoestado.sp.gov.br/web/acervo/solicitacao_certidoes/imigracao</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>Molto alta: ingressi al porto di Buenos Aires 1882-1937, serie UNESCO Memoria del Mundo, oltre 4 milioni di ingressi in 808 libri</x:v>
+        <x:v>Molto alta: Hospedaria, Porto di Santos, nuclei coloniali, documenti di immigrazione e colonizzazione</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>Buscador ufficiale pubblico: la pagina indica ricerca per date, nome, cognome e nave, con possibilita di scaricare una constancia PDF e, se digitalizzato, il PDF del libro completo. I termini generali Argentina.gob.ar indicano accesso libero/gratuito e contenuti CC BY 4.0 salvo diversa indicazione; non emergono pero API/IIIF o endpoint ufficiali documentati per automazione</x:v>
+        <x:v>Fonte ufficiale molto rilevante, ma l'acervo digitalizzato rimanda a registrazione/login e la pagina dei nuclei coloniali contiene avviso di servizio con login; la riproduzione e soggetta a credito, termini di responsabilita e valutazioni su diritto/autorizzazione. Nessun endpoint no-login/API/IIIF stabile verificato nel primo controllo</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>B - candidato forte per futura capability metadata/PDF; per ora link assistito, no download diretto finche non viene validato un endpoint pubblico stabile con fixture</x:v>
+        <x:v>C - link/manuale e discovery; download diretto escluso finche non emerge una risorsa pubblica no-login con licenza e tecnica stabili</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="607.2000122070312" hidden="0" customHeight="1">
       <x:c r="A26" s="10" t="str">
-        <x:v>cemla_buscador</x:v>
+        <x:v>arquivo_nacional_br_sian</x:v>
       </x:c>
       <x:c r="B26" s="10" t="str">
-        <x:v>CEMLA buscador inmigrantes</x:v>
+        <x:v>Arquivo Nacional do Brasil / SIAN</x:v>
       </x:c>
       <x:c r="C26" s="10" t="str">
-        <x:v>Argentina / diaspora italiana</x:v>
+        <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
-        <x:v>https://cemla.com/; https://www.cemla.com/buscador/; https://cemla.com/faqs/; https://cemla.com/contacto/; https://cemla.com/terms-and-conditions/</x:v>
+        <x:v>https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/a-imigracao-italiana-e-o-acervo-do-an; https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/quer-pesquisar-no-arquivo-nacional-acesse-o-sian; https://www.gov.br/arquivonacional/pt-br/servicos/acervos/copy_of_acervos-mais-consultados/entrada-de-estrangeiros; https://www.gov.br/arquivonacional/pt-br/servicos/bases-de-dados/bases</x:v>
       </x:c>
       <x:c r="E26" s="10" t="str">
-        <x:v>Alta: arrivi di immigrati in Argentina, con dati fino al 1960 e forte utilita per famiglie italiane</x:v>
+        <x:v>Alta: ingresso di stranieri, vapori, acervo nazionale, Porto di Rio de Janeiro e Porto di Santos</x:v>
       </x:c>
       <x:c r="F26" s="10" t="str">
-        <x:v>Fonte privata/non governativa molto usata; le FAQ chiariscono che CEMLA espone solo i dati presenti nel buscador, indica i campi disponibili e rimanda al certificato via email. Il buscador e incorporato come iframe, non espone API/IIIF o endpoint documentati, la pagina termini e un placeholder generico e il flusso pubblico richiede validazione tipo CAPTCHA</x:v>
+        <x:v>SIAN e molto rilevante e offre documenti digitalizzati senza costo, ma le fonti ufficiali richiedono cadastro/login; la pagina SIAN espone anche controllo anti-spam/umano. La base separata Entrada de Estrangeiros - Porto do Rio de Janeiro e utile come ricerca nominale/dichiarazione, ma non e ancora un endpoint immagini/API verificato</x:v>
       </x:c>
       <x:c r="G26" s="10" t="str">
-        <x:v>C - solo link/manuale; no download diretto e no interrogazione automatica senza autorizzazione/API esplicita</x:v>
+        <x:v>C - link/manuale e discovery; non integrare download diretto SIAN per login/challenge. Rivalutare separatamente la base Rio solo se emerge un accesso pubblico documentato e testabile</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="739.2000122070312" hidden="0" customHeight="1">
       <x:c r="A27" s="10" t="str">
-        <x:v>agn_colombia_dataviva</x:v>
+        <x:v>agn_argentina_inmigrantes</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Archivo General de la Nacion Colombia - DataViva</x:v>
+        <x:v>Archivo General de la Nacion Argentina - buscador inmigrantes</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
-        <x:v>Colombia / diaspora italiana</x:v>
+        <x:v>Argentina / diaspora italiana</x:v>
       </x:c>
       <x:c r="D27" s="10" t="str">
-        <x:v>https://www.archivogeneral.gov.co/agn/home/; https://dataviva.archivogeneral.gov.co/; https://www.datos.gov.co/Cultura/DATAVIVA/r5h9-7h58; https://www.archivogeneral.gov.co/dataviva-da-un-paso-historico-hacia-los-datos-abiertos-en-colombia; https://www.archivogeneral.gov.co/terminos-y-condiciones; https://www.archivogeneral.gov.co/sites/default/files/2025-07/MANUAL_DATAVIVA.pdf</x:v>
+        <x:v>https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion; https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion/consulta-de-antecedentes-migratorios; https://www.argentina.gob.ar/noticias/el-archivo-general-de-la-nacion-es-memoria-del-mundo; https://www.argentina.gob.ar/terminos-y-condiciones; https://www.unesco.org/es/memory-world/lac/passengers-entry-books-sea-1882-1937-national-registry-migrations-documentary-fond</x:v>
       </x:c>
       <x:c r="E27" s="10" t="str">
-        <x:v>Media-alta: documenti storici digitalizzati, possibili fondi migrazione e contesto per presenze italiane in Colombia</x:v>
+        <x:v>Molto alta: ingressi al porto di Buenos Aires 1882-1937, serie UNESCO Memoria del Mundo, oltre 4 milioni di ingressi in 808 libri</x:v>
       </x:c>
       <x:c r="F27" s="10" t="str">
-        <x:v>Candidato tecnico forte per metadata/discovery: il dataset ufficiale Datos Abiertos Colombia dichiara DataViva come applicazione AGN per consulta, visualizzazione e descarga di piu di 25 milioni di immagini, con accesso OData/Socrata e dati aggiornati nel 2026. Tuttavia i termini generali AGN sono restrittivi su riproduzione/copia/distribuzione dei contenuti; distinguere metadati open data da immagini/documenti e verificare per item prima di qualunque download</x:v>
+        <x:v>Buscador ufficiale pubblico: la pagina indica ricerca per date, nome, cognome e nave, con possibilita di scaricare una constancia PDF e, se digitalizzato, il PDF del libro completo. I termini generali Argentina.gob.ar indicano accesso libero/gratuito e contenuti CC BY 4.0 salvo diversa indicazione; non emergono pero API/IIIF o endpoint ufficiali documentati per automazione</x:v>
       </x:c>
       <x:c r="G27" s="10" t="str">
-        <x:v>B - forte per futura integrazione metadata/API; download immagini/PDF solo con policy specifica, range esplicito e fixture stabile</x:v>
+        <x:v>B - candidato forte per futura capability metadata/PDF; per ora link assistito, no download diretto finche non viene validato un endpoint pubblico stabile con fixture</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A28" s="10" t="str">
-        <x:v>nara_catalog</x:v>
+        <x:v>cemla_buscador</x:v>
       </x:c>
       <x:c r="B28" s="10" t="str">
-        <x:v>National Archives Catalog / NARA API</x:v>
+        <x:v>CEMLA buscador inmigrantes</x:v>
       </x:c>
       <x:c r="C28" s="10" t="str">
-        <x:v>Stati Uniti / diaspora italiana</x:v>
+        <x:v>Argentina / diaspora italiana</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
-        <x:v>https://www.archives.gov/research/catalog/help/api; https://www.archives.gov/research/immigration/overview</x:v>
+        <x:v>https://cemla.com/; https://www.cemla.com/buscador/; https://cemla.com/faqs/; https://cemla.com/contacto/; https://cemla.com/terms-and-conditions/</x:v>
       </x:c>
       <x:c r="E28" s="10" t="str">
-        <x:v>Alta: naturalizzazioni, immigrazione, passenger records, A-files</x:v>
+        <x:v>Alta: arrivi di immigrati in Argentina, con dati fino al 1960 e forte utilita per famiglie italiane</x:v>
       </x:c>
       <x:c r="F28" s="10" t="str">
-        <x:v>API ufficiale per dati pubblici del Catalog; disponibilita immagini e diritti variano per record</x:v>
+        <x:v>Fonte privata/non governativa molto usata; le FAQ chiariscono che CEMLA espone solo i dati presenti nel buscador, indica i campi disponibili e rimanda al certificato via email. Il buscador e incorporato come iframe, non espone API/IIIF o endpoint documentati, la pagina termini e un placeholder generico e il flusso pubblico richiede validazione tipo CAPTCHA</x:v>
       </x:c>
       <x:c r="G28" s="10" t="str">
-        <x:v>A/B - candidato forte per metadata/record pubblici</x:v>
+        <x:v>C - solo link/manuale; no download diretto e no interrogazione automatica senza autorizzazione/API esplicita</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A29" s="10" t="str">
-        <x:v>loc_chronicling_america</x:v>
+        <x:v>agn_colombia_dataviva</x:v>
       </x:c>
       <x:c r="B29" s="10" t="str">
-        <x:v>Library of Congress - Chronicling America / loc.gov API</x:v>
+        <x:v>Archivo General de la Nacion Colombia - DataViva</x:v>
       </x:c>
       <x:c r="C29" s="10" t="str">
-        <x:v>Stati Uniti / contesto diaspora</x:v>
+        <x:v>Colombia / diaspora italiana</x:v>
       </x:c>
       <x:c r="D29" s="10" t="str">
-        <x:v>https://www.loc.gov/apis/additional-apis/chronicling-america-api/</x:v>
+        <x:v>https://www.archivogeneral.gov.co/agn/home/; https://dataviva.archivogeneral.gov.co/; https://www.datos.gov.co/Cultura/DATAVIVA/r5h9-7h58; https://www.archivogeneral.gov.co/dataviva-da-un-paso-historico-hacia-los-datos-abiertos-en-colombia; https://www.archivogeneral.gov.co/terminos-y-condiciones; https://www.archivogeneral.gov.co/sites/default/files/2025-07/MANUAL_DATAVIVA.pdf</x:v>
       </x:c>
       <x:c r="E29" s="10" t="str">
-        <x:v>Media: giornali storici utili per contesto familiare, non atti vitali</x:v>
+        <x:v>Media-alta: documenti storici digitalizzati, possibili fondi migrazione e contesto per presenze italiane in Colombia</x:v>
       </x:c>
       <x:c r="F29" s="10" t="str">
-        <x:v>API ufficiale; utile come modulo di ricerca contestuale piu che downloader genealogico primario</x:v>
+        <x:v>Candidato tecnico forte per metadata/discovery: il dataset ufficiale Datos Abiertos Colombia dichiara DataViva come applicazione AGN per consulta, visualizzazione e descarga di piu di 25 milioni di immagini, con accesso OData/Socrata e dati aggiornati nel 2026. Tuttavia i termini generali AGN sono restrittivi su riproduzione/copia/distribuzione dei contenuti; distinguere metadati open data da immagini/documenti e verificare per item prima di qualunque download</x:v>
       </x:c>
       <x:c r="G29" s="10" t="str">
-        <x:v>B - valutare dopo fonti archivistiche</x:v>
+        <x:v>B - forte per futura integrazione metadata/API; download immagini/PDF solo con policy specifica, range esplicito e fixture stabile</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="132" hidden="0" customHeight="1">
       <x:c r="A30" s="10" t="str">
-        <x:v>naa_recordsearch</x:v>
+        <x:v>nara_catalog</x:v>
       </x:c>
       <x:c r="B30" s="10" t="str">
-        <x:v>National Archives of Australia - RecordSearch passenger arrivals</x:v>
+        <x:v>National Archives Catalog / NARA API</x:v>
       </x:c>
       <x:c r="C30" s="10" t="str">
-        <x:v>Australia / diaspora italiana</x:v>
+        <x:v>Stati Uniti / diaspora italiana</x:v>
       </x:c>
       <x:c r="D30" s="10" t="str">
-        <x:v>https://www.naa.gov.au/explore-collection/immigration-and-citizenship/passenger-arrival-records</x:v>
+        <x:v>https://www.archives.gov/research/catalog/help/api; https://www.archives.gov/research/immigration/overview</x:v>
       </x:c>
       <x:c r="E30" s="10" t="str">
-        <x:v>Alta: arrivi passeggeri 1898-1972, dati migratori</x:v>
+        <x:v>Alta: naturalizzazioni, immigrazione, passenger records, A-files</x:v>
       </x:c>
       <x:c r="F30" s="10" t="str">
-        <x:v>Fonte ufficiale e molto rilevante; API non confermata, diritti/download da verificare</x:v>
+        <x:v>API ufficiale per dati pubblici del Catalog; disponibilita immagini e diritti variano per record</x:v>
       </x:c>
       <x:c r="G30" s="10" t="str">
-        <x:v>B/C - candidato prioritario, inizialmente link assistito</x:v>
+        <x:v>A/B - candidato forte per metadata/record pubblici</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="237.60000610351562" hidden="0" customHeight="1">
       <x:c r="A31" s="10" t="str">
-        <x:v>papers_past_digitalnz</x:v>
+        <x:v>loc_chronicling_america</x:v>
       </x:c>
       <x:c r="B31" s="10" t="str">
-        <x:v>Papers Past / DigitalNZ API</x:v>
+        <x:v>Library of Congress - Chronicling America / loc.gov API</x:v>
       </x:c>
       <x:c r="C31" s="10" t="str">
-        <x:v>Nuova Zelanda / diaspora italiana</x:v>
+        <x:v>Stati Uniti / contesto diaspora</x:v>
       </x:c>
       <x:c r="D31" s="10" t="str">
-        <x:v>https://natlib.govt.nz/about-us/open-data/papers-past-metadata/papers-past-data-using-the-digitalnz-api; https://paperspast.natlib.govt.nz/help/using-papers-past-material</x:v>
+        <x:v>https://www.loc.gov/apis/additional-apis/chronicling-america-api/</x:v>
       </x:c>
       <x:c r="E31" s="10" t="str">
-        <x:v>Media: giornali e avvisi utili per tracce migratorie e familiari</x:v>
+        <x:v>Media: giornali storici utili per contesto familiare, non atti vitali</x:v>
       </x:c>
       <x:c r="F31" s="10" t="str">
-        <x:v>API metadata ufficiale via DigitalNZ; immagini/testi e copyright da verificare per item</x:v>
+        <x:v>API ufficiale; utile come modulo di ricerca contestuale piu che downloader genealogico primario</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>B - candidato per ricerca contestuale</x:v>
+        <x:v>B - valutare dopo fonti archivistiche</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A32" s="10" t="str">
-        <x:v>francearchives</x:v>
+        <x:v>naa_recordsearch</x:v>
       </x:c>
       <x:c r="B32" s="10" t="str">
-        <x:v>FranceArchives open data</x:v>
+        <x:v>National Archives of Australia - RecordSearch passenger arrivals</x:v>
       </x:c>
       <x:c r="C32" s="10" t="str">
-        <x:v>Francia / diaspora italiana</x:v>
+        <x:v>Australia / diaspora italiana</x:v>
       </x:c>
       <x:c r="D32" s="10" t="str">
-        <x:v>https://francearchives.gouv.fr/fr/open_data</x:v>
+        <x:v>https://www.naa.gov.au/explore-collection/immigration-and-citizenship/passenger-arrival-records</x:v>
       </x:c>
       <x:c r="E32" s="10" t="str">
-        <x:v>Alta per ricerche in Francia e migrazioni confinanti</x:v>
+        <x:v>Alta: arrivi passeggeri 1898-1972, dati migratori</x:v>
       </x:c>
       <x:c r="F32" s="10" t="str">
-        <x:v>Dati aperti e aggregazione di inventari; immagini e archivi dipartimentali dipendono dai provider</x:v>
+        <x:v>Fonte ufficiale e molto rilevante; API non confermata, diritti/download da verificare</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
-        <x:v>B - ottimo per discovery, download solo per provider verificati</x:v>
+        <x:v>B/C - candidato prioritario, inizialmente link assistito</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="224.39999389648438" hidden="0" customHeight="1">
       <x:c r="A33" s="10" t="str">
-        <x:v>belgium_state_archives</x:v>
+        <x:v>papers_past_digitalnz</x:v>
       </x:c>
       <x:c r="B33" s="10" t="str">
-        <x:v>State Archives of Belgium / AGATHA</x:v>
+        <x:v>Papers Past / DigitalNZ API</x:v>
       </x:c>
       <x:c r="C33" s="10" t="str">
-        <x:v>Belgio / diaspora italiana</x:v>
+        <x:v>Nuova Zelanda / diaspora italiana</x:v>
       </x:c>
       <x:c r="D33" s="10" t="str">
-        <x:v>https://archives.brussels.be/genealogy; https://news.belgium.be/fr/registres-paroissiaux-et-de-letat-civil-consultables-en-ligne-gratuitement</x:v>
+        <x:v>https://natlib.govt.nz/about-us/open-data/papers-past-metadata/papers-past-data-using-the-digitalnz-api; https://paperspast.natlib.govt.nz/help/using-papers-past-material</x:v>
       </x:c>
       <x:c r="E33" s="10" t="str">
-        <x:v>Alta: stato civile e registri parrocchiali</x:v>
+        <x:v>Media: giornali e avvisi utili per tracce migratorie e familiari</x:v>
       </x:c>
       <x:c r="F33" s="10" t="str">
-        <x:v>Consultazione gratuita ma storicamente richiede account/login per archivi online; non automatizzare accessi autenticati</x:v>
+        <x:v>API metadata ufficiale via DigitalNZ; immagini/testi e copyright da verificare per item</x:v>
       </x:c>
       <x:c r="G33" s="10" t="str">
-        <x:v>C - link/manuale, no integrazione diretta se login necessario</x:v>
+        <x:v>B - candidato per ricerca contestuale</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="198" hidden="0" customHeight="1">
       <x:c r="A34" s="10" t="str">
-        <x:v>deutsche_digitale_bibliothek</x:v>
+        <x:v>francearchives</x:v>
       </x:c>
       <x:c r="B34" s="10" t="str">
-        <x:v>Deutsche Digitale Bibliothek / DDB API</x:v>
+        <x:v>FranceArchives open data</x:v>
       </x:c>
       <x:c r="C34" s="10" t="str">
-        <x:v>Germania / diaspora italiana</x:v>
+        <x:v>Francia / diaspora italiana</x:v>
       </x:c>
       <x:c r="D34" s="10" t="str">
-        <x:v>https://www.deutsche-digitale-bibliothek.de/content/api-nutzungsbedingungen?lang=en; https://labs.deutsche-digitale-bibliothek.de/app/ddbapi/</x:v>
+        <x:v>https://francearchives.gouv.fr/fr/open_data</x:v>
       </x:c>
       <x:c r="E34" s="10" t="str">
-        <x:v>Media-alta: aggregatore culturale/archivistico tedesco</x:v>
+        <x:v>Alta per ricerche in Francia e migrazioni confinanti</x:v>
       </x:c>
       <x:c r="F34" s="10" t="str">
-        <x:v>API ufficiale ma richiede API key; diritti e contenuti digitali dipendono dai provider</x:v>
+        <x:v>Dati aperti e aggregazione di inventari; immagini e archivi dipartimentali dipendono dai provider</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
-        <x:v>B/C - metadata possibile, immagini solo item-by-item</x:v>
+        <x:v>B - ottimo per discovery, download solo per provider verificati</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A35" s="10" t="str">
-        <x:v>austrian_state_archives_ais</x:v>
+        <x:v>belgium_state_archives</x:v>
       </x:c>
       <x:c r="B35" s="10" t="str">
-        <x:v>Oesterreichisches Staatsarchiv - AIS</x:v>
+        <x:v>State Archives of Belgium / AGATHA</x:v>
       </x:c>
       <x:c r="C35" s="10" t="str">
-        <x:v>Austria / area asburgica</x:v>
+        <x:v>Belgio / diaspora italiana</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
-        <x:v>https://www.oesta.gv.at/benutzung/Recherche-zu-Hause/recherche/bestande-ais.html; https://www.statearchives.gv.at/user-information/holdings.html</x:v>
+        <x:v>https://archives.brussels.be/genealogy; https://news.belgium.be/fr/registres-paroissiaux-et-de-letat-civil-consultables-en-ligne-gratuitement</x:v>
       </x:c>
       <x:c r="E35" s="10" t="str">
-        <x:v>Alta per Lombardo-Veneto, Trentino-Alto Adige, Friuli Venezia Giulia e fonti militari/asburgiche</x:v>
+        <x:v>Alta: stato civile e registri parrocchiali</x:v>
       </x:c>
       <x:c r="F35" s="10" t="str">
-        <x:v>Sistema ufficiale di ricerca; utile per discovery e ordinazioni, non ancora candidato downloader</x:v>
+        <x:v>Consultazione gratuita ma storicamente richiede account/login per archivi online; non automatizzare accessi autenticati</x:v>
       </x:c>
       <x:c r="G35" s="10" t="str">
-        <x:v>C - link/discovery assistito</x:v>
+        <x:v>C - link/manuale, no integrazione diretta se login necessario</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="264" hidden="0" customHeight="1">
       <x:c r="A36" s="10" t="str">
+        <x:v>deutsche_digitale_bibliothek</x:v>
+      </x:c>
+      <x:c r="B36" s="10" t="str">
+        <x:v>Deutsche Digitale Bibliothek / DDB API</x:v>
+      </x:c>
+      <x:c r="C36" s="10" t="str">
+        <x:v>Germania / diaspora italiana</x:v>
+      </x:c>
+      <x:c r="D36" s="10" t="str">
+        <x:v>https://www.deutsche-digitale-bibliothek.de/content/api-nutzungsbedingungen?lang=en; https://labs.deutsche-digitale-bibliothek.de/app/ddbapi/</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="str">
+        <x:v>Media-alta: aggregatore culturale/archivistico tedesco</x:v>
+      </x:c>
+      <x:c r="F36" s="10" t="str">
+        <x:v>API ufficiale ma richiede API key; diritti e contenuti digitali dipendono dai provider</x:v>
+      </x:c>
+      <x:c r="G36" s="10" t="str">
+        <x:v>B/C - metadata possibile, immagini solo item-by-item</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>austrian_state_archives_ais</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>Oesterreichisches Staatsarchiv - AIS</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>Austria / area asburgica</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>https://www.oesta.gv.at/benutzung/Recherche-zu-Hause/recherche/bestande-ais.html; https://www.statearchives.gv.at/user-information/holdings.html</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>Alta per Lombardo-Veneto, Trentino-Alto Adige, Friuli Venezia Giulia e fonti militari/asburgiche</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>Sistema ufficiale di ricerca; utile per discovery e ordinazioni, non ancora candidato downloader</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>C - link/discovery assistito</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
         <x:v>anno_onb</x:v>
       </x:c>
-      <x:c r="B36" s="10" t="str">
+      <x:c r="B38" t="str">
         <x:v>ANNO - AustriaN Newspapers Online</x:v>
       </x:c>
-      <x:c r="C36" s="10" t="str">
+      <x:c r="C38" t="str">
         <x:v>Austria / area asburgica</x:v>
       </x:c>
-      <x:c r="D36" s="10" t="str">
+      <x:c r="D38" t="str">
         <x:v>https://dbis.ur.de/detail.php?bib_id=FUH&amp;lang=en&amp;titel_id=2012; https://www.bundeskanzleramt.gv.at/en/services/federal-administrative-library/databases/general-access-databases.html</x:v>
       </x:c>
-      <x:c r="E36" s="10" t="str">
+      <x:c r="E38" t="str">
         <x:v>Media: giornali storici per contesto migratorio, militare e civile</x:v>
       </x:c>
-      <x:c r="F36" s="10" t="str">
+      <x:c r="F38" t="str">
         <x:v>Fonte pubblica importante; API ufficiale non confermata nel primo passaggio, evitare scraping massivo</x:v>
       </x:c>
-      <x:c r="G36" s="10" t="str">
+      <x:c r="G38" t="str">
         <x:v>C/B - rivalutare se emerge API stabile o download consentito</x:v>
       </x:c>
     </x:row>

</xml_diff>